<commit_message>
Update Java24 PhuocDung Database Design 20.06.2025
</commit_message>
<xml_diff>
--- a/Java24 PhuocDung Database design.xlsx
+++ b/Java24 PhuocDung Database design.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\java24\3. Database\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9A19BADF-560D-45FE-9F18-9EE3E0636F3D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{69F4B9A1-5E00-48EB-A26B-ED2326BB02F7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,16 +25,109 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1" uniqueCount="1">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="32">
   <si>
     <t>MatHang</t>
+  </si>
+  <si>
+    <t>MaMH</t>
+  </si>
+  <si>
+    <t>Kichthuoc(s)</t>
+  </si>
+  <si>
+    <t>GiaBan</t>
+  </si>
+  <si>
+    <t>GiaMua</t>
+  </si>
+  <si>
+    <t>LoaiMatHang</t>
+  </si>
+  <si>
+    <t>ChatLieu(s)</t>
+  </si>
+  <si>
+    <t>MauSac(s)</t>
+  </si>
+  <si>
+    <t>HinhAnh(s)</t>
+  </si>
+  <si>
+    <t>THIẾT KẾ DATABASE - WEBSITE QUẢN LÍ CỬA HÀNG THỜI TRANG</t>
+  </si>
+  <si>
+    <t>KhachHang</t>
+  </si>
+  <si>
+    <t>DonHang</t>
+  </si>
+  <si>
+    <t>TaiKhoan</t>
+  </si>
+  <si>
+    <t>Admin</t>
+  </si>
+  <si>
+    <t>HoTen</t>
+  </si>
+  <si>
+    <t>GioiTinh</t>
+  </si>
+  <si>
+    <t>NamSinh</t>
+  </si>
+  <si>
+    <t>LichSuMuaHang</t>
+  </si>
+  <si>
+    <t>DiaChi</t>
+  </si>
+  <si>
+    <t>TenTaiKhoan</t>
+  </si>
+  <si>
+    <t>MatKhau</t>
+  </si>
+  <si>
+    <t>Email</t>
+  </si>
+  <si>
+    <t>SanPham</t>
+  </si>
+  <si>
+    <t>SoLuong</t>
+  </si>
+  <si>
+    <t>GiamGia</t>
+  </si>
+  <si>
+    <t>TenAdmin</t>
+  </si>
+  <si>
+    <t>ChucVu</t>
+  </si>
+  <si>
+    <t>QuyenHan</t>
+  </si>
+  <si>
+    <t>PhiVanChuyen</t>
+  </si>
+  <si>
+    <t>NgayGiao</t>
+  </si>
+  <si>
+    <t>PhuongThucThanh Toan</t>
+  </si>
+  <si>
+    <t>KhoHang</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -42,16 +135,35 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -59,12 +171,37 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -345,15 +482,206 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="C3"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="C1:L11"/>
+  <sheetFormatPr defaultColWidth="16.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="5" width="16.85546875" style="2"/>
+    <col min="6" max="6" width="26.85546875" style="2" customWidth="1"/>
+    <col min="7" max="7" width="16.85546875" style="2"/>
+    <col min="8" max="8" width="30.42578125" style="2" customWidth="1"/>
+    <col min="9" max="16384" width="16.85546875" style="2"/>
+  </cols>
   <sheetData>
-    <row r="3" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C3" t="s">
+    <row r="1" spans="3:12" x14ac:dyDescent="0.25">
+      <c r="E1" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="F1" s="4"/>
+      <c r="G1" s="4"/>
+      <c r="H1" s="4"/>
+    </row>
+    <row r="3" spans="3:12" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C3" s="1" t="s">
         <v>0</v>
       </c>
+      <c r="D3" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E3" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="F3" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="G3" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="H3" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="I3" s="1"/>
+      <c r="J3" s="1"/>
+      <c r="K3" s="1"/>
+      <c r="L3" s="1"/>
+    </row>
+    <row r="4" spans="3:12" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C4" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="D4" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="E4" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="F4" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="G4" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="H4" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="I4" s="3"/>
+      <c r="J4" s="3"/>
+      <c r="K4" s="3"/>
+      <c r="L4" s="3"/>
+    </row>
+    <row r="5" spans="3:12" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C5" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="D5" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="E5" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="F5" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="G5" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="H5" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="I5" s="3"/>
+      <c r="J5" s="3"/>
+      <c r="K5" s="3"/>
+      <c r="L5" s="3"/>
+    </row>
+    <row r="6" spans="3:12" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C6" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="D6" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="E6" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="F6" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="G6" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="H6" s="3"/>
+      <c r="I6" s="3"/>
+      <c r="J6" s="3"/>
+      <c r="K6" s="3"/>
+      <c r="L6" s="3"/>
+    </row>
+    <row r="7" spans="3:12" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C7" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="D7" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="E7" s="3"/>
+      <c r="F7" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="G7" s="3"/>
+      <c r="H7" s="3"/>
+      <c r="I7" s="3"/>
+      <c r="J7" s="3"/>
+      <c r="K7" s="3"/>
+      <c r="L7" s="3"/>
+    </row>
+    <row r="8" spans="3:12" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C8" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="D8" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="E8" s="3"/>
+      <c r="F8" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="G8" s="3"/>
+      <c r="H8" s="3"/>
+      <c r="I8" s="3"/>
+      <c r="J8" s="3"/>
+      <c r="K8" s="3"/>
+      <c r="L8" s="3"/>
+    </row>
+    <row r="9" spans="3:12" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C9" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="D9" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="E9" s="3"/>
+      <c r="F9" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="G9" s="3"/>
+      <c r="H9" s="3"/>
+      <c r="I9" s="3"/>
+      <c r="J9" s="3"/>
+      <c r="K9" s="3"/>
+      <c r="L9" s="3"/>
+    </row>
+    <row r="10" spans="3:12" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C10" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D10" s="3"/>
+      <c r="E10" s="3"/>
+      <c r="F10" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="G10" s="3"/>
+      <c r="H10" s="3"/>
+      <c r="I10" s="3"/>
+      <c r="J10" s="3"/>
+      <c r="K10" s="3"/>
+      <c r="L10" s="3"/>
+    </row>
+    <row r="11" spans="3:12" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C11" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="D11" s="3"/>
+      <c r="E11" s="3"/>
+      <c r="F11" s="3"/>
+      <c r="G11" s="3"/>
+      <c r="H11" s="3"/>
+      <c r="I11" s="3"/>
+      <c r="J11" s="3"/>
+      <c r="K11" s="3"/>
+      <c r="L11" s="3"/>
     </row>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="E1:H1"/>
+  </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>